<commit_message>
Add scripts for processing Ellingham diagram data and melting points
- Created `ellingham_v6_data.py` to transform raw data from the Ellingham diagram into a clean, structured Excel workbook.
- Introduced `ellingham_v6_melting.py` to store melting points of metals and oxides for phase change markings.
- Added `find_melting_in_v6.py` to search for melting point information in the Ellingham workbook.
- Implemented `reaktoro_test.py` to include a basic import of the Reaktoro library for future testing.
</commit_message>
<xml_diff>
--- a/data/ellingham/ellingham_data.xlsx
+++ b/data/ellingham/ellingham_data.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="6"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="oxides" sheetId="1" state="visible" r:id="rId3"/>
@@ -12725,7 +12725,7 @@
   <dimension ref="A1:H14"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="18.68"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="18.68"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13111,7 +13111,7 @@
   <dimension ref="A1:H213"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="41.08"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="41.08"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18671,7 +18671,7 @@
   <dimension ref="A1:H36"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="38.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="38.72"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19629,7 +19629,7 @@
   <dimension ref="A1:H240"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="42.2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="42.2"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -25891,7 +25891,7 @@
   <dimension ref="A1:H55"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="40.25"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="40.25"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27342,6 +27342,9 @@
   </sheetPr>
   <dimension ref="A1:H74"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="42.05"/>
+  </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">

</xml_diff>